<commit_message>
fix: add a general pipeline to run MOMA in etfl model
</commit_message>
<xml_diff>
--- a/examples/result/core_model_abundance.xlsx
+++ b/examples/result/core_model_abundance.xlsx
@@ -446,11 +446,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>EZ_PGI</t>
+          <t>EZ_ACONTb_inferred_1</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.404807046339953e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -459,7 +459,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EZ_ACALD_inferred_0</t>
+          <t>EZ_FBA_inferred_2</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -472,11 +472,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EZ_GLNS_inferred_1</t>
+          <t>EZ_dummy_enzyme</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>0.0006099892687149776</v>
       </c>
     </row>
     <row r="5">
@@ -485,7 +485,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EZ_TKT2_inferred_0</t>
+          <t>EZ_FORti_inferred_0</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -498,7 +498,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EZ_PPCK_inferred_0</t>
+          <t>EZ_NADTRHD_inferred_0</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -511,7 +511,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EZ_AKGt2r_inferred_0</t>
+          <t>EZ_ACALD_inferred_1</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -524,11 +524,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EZ_MDH</t>
+          <t>EZ_PIt2r_inferred_1</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>2.43835919951647e-06</v>
       </c>
     </row>
     <row r="9">
@@ -537,11 +537,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EZ_SUCCt2_2_inferred_0</t>
+          <t>EZ_PFL_inferred_0</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>1.414073979862304e-05</v>
       </c>
     </row>
     <row r="10">
@@ -550,11 +550,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EZ_FRD7_inferred_0</t>
+          <t>EZ_FORt2_inferred_0</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>7.058431574991063e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -563,7 +563,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EZ_TALA_inferred_0</t>
+          <t>EZ_GLUN_inferred_2</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -576,11 +576,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EZ_CS</t>
+          <t>EZ_ICDHyr</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6.966341628920187e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -589,7 +589,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EZ_PYK_inferred_1</t>
+          <t>EZ_D_LACt2_inferred_1</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -602,11 +602,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EZ_LDH_D_inferred_0</t>
+          <t>EZ_ENO</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>0.0001003887356586803</v>
       </c>
     </row>
     <row r="15">
@@ -615,7 +615,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EZ_FORti_inferred_1</t>
+          <t>EZ_GLNS_inferred_0</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -628,11 +628,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EZ_ICL_inferred_0</t>
+          <t>EZ_FUM_inferred_2</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>7.058431574991064e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -641,11 +641,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EZ_TKT1_inferred_1</t>
+          <t>EZ_PPS_inferred_0</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.35188481084382e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -654,7 +654,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>EZ_PGM_inferred_1</t>
+          <t>EZ_GLUSy_inferred_0</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -667,11 +667,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>EZ_RPE_inferred_1</t>
+          <t>EZ_PFK</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2.458681215539631e-06</v>
+        <v>2.166388760976409e-06</v>
       </c>
     </row>
     <row r="20">
@@ -680,11 +680,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EZ_FORti_inferred_0</t>
+          <t>EZ_FUM_inferred_0</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1.405608241778324e-05</v>
+        <v>7.046175539043653e-06</v>
       </c>
     </row>
     <row r="21">
@@ -693,11 +693,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>EZ_GLUt2r_inferred_0</t>
+          <t>EZ_MALS_inferred_1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>7.046175539043654e-06</v>
       </c>
     </row>
     <row r="22">
@@ -706,11 +706,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>EZ_FORt2_inferred_0</t>
+          <t>EZ_PYK_inferred_0</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>3.273636282096977e-06</v>
       </c>
     </row>
     <row r="23">
@@ -719,7 +719,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EZ_FBA_inferred_1</t>
+          <t>EZ_RPI_inferred_0</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -732,7 +732,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EZ_ACALD_inferred_1</t>
+          <t>EZ_ALCD2x_inferred_1</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -745,11 +745,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EZ_RPE_inferred_0</t>
+          <t>EZ_ACKr_inferred_0</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>8.917419321659517e-07</v>
       </c>
     </row>
     <row r="26">
@@ -758,7 +758,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>EZ_FORt2_inferred_1</t>
+          <t>EZ_FBP_inferred_0</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -771,7 +771,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EZ_GLUN_inferred_0</t>
+          <t>EZ_ALCD2x_inferred_0</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -784,7 +784,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EZ_ACKr_inferred_1</t>
+          <t>EZ_FBP_inferred_1</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -797,11 +797,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EZ_GND</t>
+          <t>EZ_FUMt2_2_inferred_0</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1.725115495602772e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -810,11 +810,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EZ_PIt2r_inferred_1</t>
+          <t>EZ_NADH16_inferred_0</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2.437032617690991e-06</v>
+        <v>3.766619369052397e-05</v>
       </c>
     </row>
     <row r="31">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EZ_ACONTb_inferred_0</t>
+          <t>EZ_ACONTa_inferred_0</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>7.058431574991063e-06</v>
+        <v>7.046175539043653e-06</v>
       </c>
     </row>
     <row r="32">
@@ -836,11 +836,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>EZ_dummy_enzyme</t>
+          <t>EZ_PGM_inferred_2</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.0006064613208340314</v>
+        <v>2.805953141811025e-05</v>
       </c>
     </row>
     <row r="33">
@@ -849,11 +849,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EZ_RPI_inferred_1</t>
+          <t>EZ_ACONTb_inferred_0</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1.961347033001902e-06</v>
+        <v>7.046175539043653e-06</v>
       </c>
     </row>
     <row r="34">
@@ -862,11 +862,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>EZ_ACONTb_inferred_1</t>
+          <t>EZ_ATPS4r</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>1.857088227899539e-05</v>
       </c>
     </row>
     <row r="35">
@@ -875,7 +875,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EZ_GLUSy_inferred_0</t>
+          <t>EZ_ME2_inferred_0</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -888,11 +888,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EZ_NADTRHD_inferred_0</t>
+          <t>EZ_RPI_inferred_1</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>1.960094889662779e-06</v>
       </c>
     </row>
     <row r="37">
@@ -901,11 +901,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>EZ_GLUDy</t>
+          <t>EZ_FORt2_inferred_1</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>7.400660736942497e-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -914,7 +914,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EZ_ICDHyr</t>
+          <t>EZ_MDH</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -927,11 +927,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EZ_FUMt2_2_inferred_0</t>
+          <t>EZ_PGL</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>4.122642122366116e-06</v>
       </c>
     </row>
     <row r="40">
@@ -940,7 +940,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EZ_ALCD2x_inferred_0</t>
+          <t>EZ_PGM_inferred_1</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -953,11 +953,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>EZ_ME2_inferred_0</t>
+          <t>EZ_AKGDH_inferred_0</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>2.798909075731698e-06</v>
       </c>
     </row>
     <row r="42">
@@ -966,11 +966,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EZ_PFK</t>
+          <t>EZ_PGK</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2.166176930262114e-06</v>
+        <v>0.0001188801592008396</v>
       </c>
     </row>
     <row r="43">
@@ -979,7 +979,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>EZ_FUM_inferred_2</t>
+          <t>EZ_ACONTa_inferred_1</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -992,11 +992,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EZ_TPI</t>
+          <t>EZ_PPCK_inferred_0</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1.672769962813522e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EZ_PPS_inferred_0</t>
+          <t>EZ_ALCD2x_inferred_2</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1018,11 +1018,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EZ_PGK</t>
+          <t>EZ_CYTBD_inferred_0</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.0001188716040119177</v>
+        <v>3.062001815148032e-05</v>
       </c>
     </row>
     <row r="47">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EZ_GLUN_inferred_2</t>
+          <t>EZ_GLNabc_inferred_0</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EZ_D_LACt2_inferred_0</t>
+          <t>EZ_PTAr_inferred_0</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1057,11 +1057,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EZ_FUM_inferred_0</t>
+          <t>EZ_CS</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>7.058431574991063e-06</v>
+        <v>6.954245495024309e-06</v>
       </c>
     </row>
     <row r="50">
@@ -1070,11 +1070,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EZ_D_LACt2_inferred_1</t>
+          <t>EZ_ADK1</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>1.528393083046343e-09</v>
       </c>
     </row>
     <row r="51">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>EZ_GLNS_inferred_0</t>
+          <t>EZ_MALS_inferred_0</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1096,11 +1096,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EZ_FBA_inferred_0</t>
+          <t>EZ_GLNS_inferred_1</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1.40266159401855e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -1109,11 +1109,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EZ_PPC</t>
+          <t>EZ_GLUDy</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>7.719863209285987e-06</v>
+        <v>7.401876820648816e-10</v>
       </c>
     </row>
     <row r="54">
@@ -1122,11 +1122,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>EZ_THD2_inferred_0</t>
+          <t>EZ_ICL_inferred_0</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0</v>
+        <v>7.046175539043654e-06</v>
       </c>
     </row>
     <row r="55">
@@ -1135,11 +1135,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EZ_MALS_inferred_1</t>
+          <t>EZ_GAPD</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>7.058431574991065e-06</v>
+        <v>4.304281626237295e-05</v>
       </c>
     </row>
     <row r="56">
@@ -1148,11 +1148,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EZ_rib</t>
+          <t>EZ_SUCOAS_inferred_0</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>7.271793563412013e-07</v>
+        <v>2.798909075731697e-06</v>
       </c>
     </row>
     <row r="57">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EZ_LDH_D_inferred_1</t>
+          <t>EZ_LDH_D_inferred_0</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -1174,11 +1174,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>EZ_rnap</t>
+          <t>EZ_GLCpts_inferred_0</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>9.726954619206719e-09</v>
+        <v>1.617527569134871e-05</v>
       </c>
     </row>
     <row r="59">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EZ_FBA_inferred_2</t>
+          <t>EZ_GLUN_inferred_1</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -1200,11 +1200,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EZ_ME1_inferred_0</t>
+          <t>EZ_TPI</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0</v>
+        <v>1.672933543198449e-05</v>
       </c>
     </row>
     <row r="61">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>EZ_ALCD2x_inferred_1</t>
+          <t>EZ_TKT1_inferred_0</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -1226,11 +1226,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EZ_FRUpts2_inferred_0</t>
+          <t>EZ_FRD7_inferred_0</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0</v>
+        <v>7.046175539043653e-06</v>
       </c>
     </row>
     <row r="63">
@@ -1239,11 +1239,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EZ_GAPD</t>
+          <t>EZ_PTAr_inferred_1</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>4.303971869397019e-05</v>
+        <v>8.917419321659515e-07</v>
       </c>
     </row>
     <row r="64">
@@ -1252,11 +1252,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>EZ_TALA_inferred_1</t>
+          <t>EZ_PPC</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1.35188481084382e-06</v>
+        <v>7.707702082092862e-06</v>
       </c>
     </row>
     <row r="65">
@@ -1265,11 +1265,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EZ_ACONTa_inferred_0</t>
+          <t>EZ_G6PDH2r</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>7.058431574991063e-06</v>
+        <v>4.89397516461526e-06</v>
       </c>
     </row>
     <row r="66">
@@ -1278,11 +1278,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EZ_PYK_inferred_0</t>
+          <t>EZ_D_LACt2_inferred_0</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>3.257640944248926e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EZ_RPI_inferred_0</t>
+          <t>EZ_ACKr_inferred_2</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -1304,11 +1304,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EZ_FBP_inferred_0</t>
+          <t>EZ_rib</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0</v>
+        <v>7.028182970753551e-07</v>
       </c>
     </row>
     <row r="69">
@@ -1317,11 +1317,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EZ_ACKr_inferred_0</t>
+          <t>EZ_TKT2_inferred_1</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>8.483837750958758e-07</v>
+        <v>1.106089536204087e-06</v>
       </c>
     </row>
     <row r="70">
@@ -1330,11 +1330,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>EZ_NADH16_inferred_0</t>
+          <t>EZ_THD2_inferred_0</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>3.773485602223082e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -1343,11 +1343,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EZ_FBP_inferred_1</t>
+          <t>EZ_PDH_inferred_0</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0</v>
+        <v>3.386168230055992e-06</v>
       </c>
     </row>
     <row r="72">
@@ -1356,11 +1356,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EZ_ATPS4r</t>
+          <t>EZ_TKT2_inferred_0</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1.862989170361976e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -1369,11 +1369,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EZ_PGM_inferred_2</t>
+          <t>EZ_PGM_inferred_0</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2.805679099977451e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -1382,11 +1382,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>EZ_AKGDH_inferred_0</t>
+          <t>EZ_PGI</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2.800692313593889e-06</v>
+        <v>1.405159101522725e-05</v>
       </c>
     </row>
     <row r="75">
@@ -1395,11 +1395,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EZ_PGL</t>
+          <t>EZ_SUCCt2_2_inferred_0</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>4.125276185137063e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>EZ_ALCD2x_inferred_2</t>
+          <t>EZ_MALt2_2_inferred_0</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EZ_ACONTa_inferred_1</t>
+          <t>EZ_AKGt2r_inferred_0</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>EZ_GLNabc_inferred_0</t>
+          <t>EZ_LDH_D_inferred_1</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -1447,11 +1447,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>EZ_CYTBD_inferred_0</t>
+          <t>EZ_rnap</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3.067642444723975e-05</v>
+        <v>3.720897709586691e-09</v>
       </c>
     </row>
     <row r="80">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>EZ_MALS_inferred_0</t>
+          <t>EZ_ACALD_inferred_0</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>EZ_PTAr_inferred_0</t>
+          <t>EZ_PYK_inferred_1</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>EZ_GLUN_inferred_1</t>
+          <t>EZ_FUM_inferred_1</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -1499,11 +1499,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>EZ_SUCOAS_inferred_0</t>
+          <t>EZ_TALA_inferred_0</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2.800692313593888e-06</v>
+        <v>1.351021555429151e-06</v>
       </c>
     </row>
     <row r="84">
@@ -1512,11 +1512,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>EZ_PTAr_inferred_1</t>
+          <t>EZ_FRUpts2_inferred_0</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>8.483837750958756e-07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -1525,11 +1525,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>EZ_G6PDH2r</t>
+          <t>EZ_ME1_inferred_0</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>4.897102052033674e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -1538,11 +1538,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>EZ_PDH_inferred_0</t>
+          <t>EZ_TALA_inferred_1</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>3.453603090567646e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87">
@@ -1551,11 +1551,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EZ_TKT2_inferred_1</t>
+          <t>EZ_SUCDi_inferred_0</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1.106796404695811e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EZ_MALt2_2_inferred_0</t>
+          <t>EZ_PIt2r_inferred_0</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -1577,11 +1577,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>EZ_TKT1_inferred_0</t>
+          <t>EZ_TKT1_inferred_1</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>0</v>
+        <v>1.351021555429151e-06</v>
       </c>
     </row>
     <row r="90">
@@ -1590,11 +1590,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EZ_SUCDi_inferred_0</t>
+          <t>EZ_FORti_inferred_1</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>0</v>
+        <v>1.414073979862305e-05</v>
       </c>
     </row>
     <row r="91">
@@ -1603,11 +1603,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EZ_PFL_inferred_0</t>
+          <t>EZ_GLUt2r_inferred_0</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1.405608241778324e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -1616,11 +1616,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>EZ_ACKr_inferred_2</t>
+          <t>EZ_FBA_inferred_0</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>0</v>
+        <v>1.402798760472141e-05</v>
       </c>
     </row>
     <row r="93">
@@ -1629,11 +1629,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EZ_PIt2r_inferred_0</t>
+          <t>EZ_RPE_inferred_1</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>0</v>
+        <v>2.457111091633238e-06</v>
       </c>
     </row>
     <row r="94">
@@ -1642,11 +1642,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>EZ_GLCpts_inferred_0</t>
+          <t>EZ_RPE_inferred_0</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1.617527569134871e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>EZ_PGM_inferred_0</t>
+          <t>EZ_FBA_inferred_1</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -1668,11 +1668,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>EZ_ADK1</t>
+          <t>EZ_GND</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1.587163132383176e-09</v>
+        <v>1.724013978444012e-05</v>
       </c>
     </row>
     <row r="97">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>EZ_FUM_inferred_1</t>
+          <t>EZ_GLUN_inferred_0</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -1694,11 +1694,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>EZ_ENO</t>
+          <t>EZ_ACKr_inferred_1</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>0.0001003789312493408</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update some MOM/PA test codes for ecYeast and ETFL model
</commit_message>
<xml_diff>
--- a/examples/result/core_model_abundance.xlsx
+++ b/examples/result/core_model_abundance.xlsx
@@ -446,11 +446,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>EZ_PGK</t>
+          <t>EZ_PIt2r_inferred_0</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4.444546807589489e-05</v>
+        <v>3.085271929387718e-06</v>
       </c>
     </row>
     <row r="3">
@@ -459,7 +459,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EZ_FUM_inferred_1</t>
+          <t>EZ_GLUN_inferred_0</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -472,11 +472,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EZ_MDH</t>
+          <t>EZ_ACALD_inferred_1</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6.434929443975906e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -485,7 +485,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EZ_FORt2_inferred_1</t>
+          <t>EZ_RPE_inferred_0</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -498,11 +498,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EZ_ICL_inferred_0</t>
+          <t>EZ_TALA_inferred_1</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1.005431696471998e-06</v>
       </c>
     </row>
     <row r="7">
@@ -511,11 +511,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EZ_GLNS_inferred_1</t>
+          <t>EZ_rnap</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>1.00982598522738e-08</v>
       </c>
     </row>
     <row r="8">
@@ -524,11 +524,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EZ_CS</t>
+          <t>EZ_PGI</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3.804548321901798e-06</v>
+        <v>4.221853848193654e-06</v>
       </c>
     </row>
     <row r="9">
@@ -537,7 +537,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EZ_LDH_D_inferred_0</t>
+          <t>EZ_FORti_inferred_1</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -550,7 +550,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EZ_FORt2_inferred_0</t>
+          <t>EZ_ME1_inferred_0</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -563,11 +563,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EZ_dummy_enzyme</t>
+          <t>EZ_FRUpts2_inferred_0</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.0006115090754412706</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -576,11 +576,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EZ_PIt2r_inferred_1</t>
+          <t>EZ_rib</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>8.757374267288781e-07</v>
       </c>
     </row>
     <row r="13">
@@ -589,11 +589,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EZ_FORti_inferred_0</t>
+          <t>EZ_SUCDi_inferred_0</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>5.775578276093037e-06</v>
       </c>
     </row>
     <row r="14">
@@ -602,7 +602,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EZ_ACALD_inferred_1</t>
+          <t>EZ_ACALD_inferred_0</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -615,7 +615,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EZ_GLUN_inferred_0</t>
+          <t>EZ_SUCCt2_2_inferred_0</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -628,7 +628,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EZ_NADTRHD_inferred_0</t>
+          <t>EZ_THD2_inferred_0</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -641,11 +641,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EZ_ACONTb_inferred_1</t>
+          <t>EZ_MDH</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>6.420251208182152e-05</v>
       </c>
     </row>
     <row r="18">
@@ -654,11 +654,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>EZ_ACKr_inferred_1</t>
+          <t>EZ_ENO</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>3.419969635669603e-05</v>
       </c>
     </row>
     <row r="19">
@@ -667,11 +667,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>EZ_ICDHyr</t>
+          <t>EZ_LDH_D_inferred_1</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3.009051854595058e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -680,11 +680,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EZ_GND</t>
+          <t>EZ_LDH_D_inferred_0</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1.361726409801756e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -693,7 +693,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>EZ_RPE_inferred_0</t>
+          <t>EZ_AKGt2r_inferred_0</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -706,7 +706,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>EZ_D_LACt2_inferred_0</t>
+          <t>EZ_ACKr_inferred_1</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -719,7 +719,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EZ_PPC</t>
+          <t>EZ_ACKr_inferred_2</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -732,11 +732,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EZ_FRD7_inferred_0</t>
+          <t>EZ_TKT2_inferred_1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>6.950794423306358e-07</v>
       </c>
     </row>
     <row r="25">
@@ -745,11 +745,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EZ_ENO</t>
+          <t>EZ_PDH_inferred_0</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3.427350998483843e-05</v>
+        <v>7.069510118598224e-06</v>
       </c>
     </row>
     <row r="26">
@@ -758,7 +758,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>EZ_PGM_inferred_1</t>
+          <t>EZ_PIt2r_inferred_1</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -771,7 +771,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EZ_PPCK_inferred_0</t>
+          <t>EZ_GLUt2r_inferred_0</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -784,7 +784,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EZ_THD2_inferred_0</t>
+          <t>EZ_FBA_inferred_1</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -797,11 +797,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EZ_rib</t>
+          <t>EZ_TKT2_inferred_0</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>7.908621629445962e-07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -810,7 +810,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EZ_LDH_D_inferred_1</t>
+          <t>EZ_MALt2_2_inferred_0</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EZ_rnap</t>
+          <t>EZ_FORt2_inferred_0</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>9.554596548736217e-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -836,7 +836,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>EZ_ME1_inferred_0</t>
+          <t>EZ_PGM_inferred_1</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -849,7 +849,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EZ_FRUpts2_inferred_0</t>
+          <t>EZ_FORt2_inferred_1</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -862,11 +862,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>EZ_SUCDi_inferred_0</t>
+          <t>EZ_CS</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>5.794392790242042e-06</v>
+        <v>3.797322871972418e-06</v>
       </c>
     </row>
     <row r="35">
@@ -875,11 +875,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EZ_TALA_inferred_1</t>
+          <t>EZ_PPC</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1.008688686247117e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -888,11 +888,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EZ_TPI</t>
+          <t>EZ_TKT1_inferred_1</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>6.132168121303484e-06</v>
+        <v>1.005431696471998e-06</v>
       </c>
     </row>
     <row r="37">
@@ -901,11 +901,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>EZ_NADH16_inferred_0</t>
+          <t>EZ_PPCK_inferred_0</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3.382436751772018e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -914,7 +914,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EZ_FBP_inferred_1</t>
+          <t>EZ_GLNS_inferred_1</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -927,11 +927,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EZ_ATPS4r</t>
+          <t>EZ_PGK</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3.041045687226646e-05</v>
+        <v>4.434403599173185e-05</v>
       </c>
     </row>
     <row r="40">
@@ -940,11 +940,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EZ_PGM_inferred_2</t>
+          <t>EZ_D_LACt2_inferred_0</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.0004639508396411812</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -953,11 +953,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>EZ_AKGDH_inferred_0</t>
+          <t>EZ_NADTRHD_inferred_0</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>7.411920359376913e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -966,11 +966,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EZ_PGL</t>
+          <t>EZ_TALA_inferred_0</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3.256302284308546e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -979,7 +979,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>EZ_ALCD2x_inferred_2</t>
+          <t>EZ_PYK_inferred_1</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -992,7 +992,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EZ_ACONTa_inferred_1</t>
+          <t>EZ_ICL_inferred_0</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1005,11 +1005,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EZ_GLNabc_inferred_0</t>
+          <t>EZ_TPI</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>6.118502489390491e-06</v>
       </c>
     </row>
     <row r="46">
@@ -1018,11 +1018,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EZ_CYTBD_inferred_0</t>
+          <t>EZ_FRD7_inferred_0</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>3.961876030796222e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1031,11 +1031,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EZ_PTAr_inferred_0</t>
+          <t>EZ_dummy_enzyme</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>0.0006028218854288184</v>
       </c>
     </row>
     <row r="48">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EZ_GLUN_inferred_1</t>
+          <t>EZ_ACONTb_inferred_1</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1057,11 +1057,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EZ_SUCOAS_inferred_0</t>
+          <t>EZ_GND</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>7.411920359376913e-06</v>
+        <v>1.357328161602392e-05</v>
       </c>
     </row>
     <row r="50">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EZ_PTAr_inferred_1</t>
+          <t>EZ_FORti_inferred_0</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>EZ_G6PDH2r</t>
+          <t>EZ_ICDHyr</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3.865545937501758e-06</v>
+        <v>3.003337180560004e-05</v>
       </c>
     </row>
     <row r="52">
@@ -1096,11 +1096,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EZ_PFL_inferred_0</t>
+          <t>EZ_RPE_inferred_1</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0</v>
+        <v>1.700511138802634e-06</v>
       </c>
     </row>
     <row r="53">
@@ -1109,11 +1109,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EZ_TKT2_inferred_1</t>
+          <t>EZ_ACONTb_inferred_0</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>6.973287918340679e-07</v>
+        <v>3.847520705659172e-06</v>
       </c>
     </row>
     <row r="54">
@@ -1122,11 +1122,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>EZ_MALt2_2_inferred_0</t>
+          <t>EZ_RPI_inferred_1</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0</v>
+        <v>1.77718576445732e-06</v>
       </c>
     </row>
     <row r="55">
@@ -1135,11 +1135,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EZ_PGI</t>
+          <t>EZ_MALS_inferred_1</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>4.229292111440625e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -1148,11 +1148,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EZ_ACALD_inferred_0</t>
+          <t>EZ_ACONTa_inferred_0</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0</v>
+        <v>3.847520705659172e-06</v>
       </c>
     </row>
     <row r="57">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EZ_TKT2_inferred_0</t>
+          <t>EZ_FUMt2_2_inferred_0</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>EZ_GLNS_inferred_0</t>
+          <t>EZ_ACKr_inferred_0</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -1187,11 +1187,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EZ_AKGt2r_inferred_0</t>
+          <t>EZ_PGL</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>3.245784734266589e-06</v>
       </c>
     </row>
     <row r="60">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EZ_GLUN_inferred_2</t>
+          <t>EZ_RPI_inferred_0</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>EZ_SUCCt2_2_inferred_0</t>
+          <t>EZ_FBP_inferred_0</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -1226,11 +1226,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EZ_D_LACt2_inferred_1</t>
+          <t>EZ_NADH16_inferred_0</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0</v>
+        <v>3.37407550992011e-05</v>
       </c>
     </row>
     <row r="63">
@@ -1239,11 +1239,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EZ_TALA_inferred_0</t>
+          <t>EZ_AKGDH_inferred_0</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>0</v>
+        <v>7.393105845227908e-06</v>
       </c>
     </row>
     <row r="64">
@@ -1252,11 +1252,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>EZ_FBA_inferred_0</t>
+          <t>EZ_MALS_inferred_0</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>5.14198419569311e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EZ_PYK_inferred_1</t>
+          <t>EZ_FBP_inferred_1</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -1278,11 +1278,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EZ_MALS_inferred_1</t>
+          <t>EZ_ATPS4r</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0</v>
+        <v>3.033307109463731e-05</v>
       </c>
     </row>
     <row r="67">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EZ_FORti_inferred_1</t>
+          <t>EZ_GLNabc_inferred_0</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -1304,11 +1304,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EZ_TKT1_inferred_1</t>
+          <t>EZ_PGM_inferred_2</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1.008688686247117e-06</v>
+        <v>0.000477674551765057</v>
       </c>
     </row>
     <row r="69">
@@ -1317,11 +1317,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EZ_FUM_inferred_2</t>
+          <t>EZ_G6PDH2r</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>5.794392790242041e-06</v>
+        <v>3.853060587774532e-06</v>
       </c>
     </row>
     <row r="70">
@@ -1330,11 +1330,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>EZ_RPE_inferred_1</t>
+          <t>EZ_PFL_inferred_0</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1.706017478081185e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -1343,11 +1343,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EZ_PIt2r_inferred_0</t>
+          <t>EZ_D_LACt2_inferred_1</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>3.105455241279016e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EZ_GLUt2r_inferred_0</t>
+          <t>EZ_ALCD2x_inferred_2</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EZ_FBA_inferred_1</t>
+          <t>EZ_ACONTa_inferred_1</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -1382,11 +1382,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>EZ_MALS_inferred_0</t>
+          <t>EZ_CYTBD_inferred_0</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0</v>
+        <v>3.951633337529414e-05</v>
       </c>
     </row>
     <row r="75">
@@ -1395,11 +1395,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EZ_PDH_inferred_0</t>
+          <t>EZ_PTAr_inferred_1</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>7.08729212028951e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>EZ_FUMt2_2_inferred_0</t>
+          <t>EZ_ALCD2x_inferred_1</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EZ_FUM_inferred_0</t>
+          <t>EZ_PGM_inferred_0</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -1434,11 +1434,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>EZ_RPI_inferred_1</t>
+          <t>EZ_PTAr_inferred_0</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1.782948456924664e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -1447,11 +1447,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>EZ_ALCD2x_inferred_0</t>
+          <t>EZ_SUCOAS_inferred_0</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0</v>
+        <v>7.393105845227907e-06</v>
       </c>
     </row>
     <row r="80">
@@ -1460,11 +1460,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>EZ_ME2_inferred_0</t>
+          <t>EZ_GLUN_inferred_1</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3.985352653359985e-07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -1473,11 +1473,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>EZ_PFK</t>
+          <t>EZ_FBA_inferred_2</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>7.940937135500915e-07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -1486,11 +1486,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>EZ_ACONTa_inferred_0</t>
+          <t>EZ_FBA_inferred_0</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>3.854841670757026e-06</v>
+        <v>5.130525204039465e-06</v>
       </c>
     </row>
     <row r="83">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>EZ_PGM_inferred_0</t>
+          <t>EZ_GLNS_inferred_0</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -1512,11 +1512,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>EZ_PYK_inferred_0</t>
+          <t>EZ_GLUDy</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1.969131997418083e-06</v>
+        <v>7.986642087688413e-10</v>
       </c>
     </row>
     <row r="85">
@@ -1525,11 +1525,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>EZ_GLUSy_inferred_0</t>
+          <t>EZ_GAPD</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0</v>
+        <v>1.605559923838567e-05</v>
       </c>
     </row>
     <row r="86">
@@ -1538,11 +1538,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>EZ_PPS_inferred_0</t>
+          <t>EZ_GLCpts_inferred_0</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>0</v>
+        <v>7.144902622007886e-06</v>
       </c>
     </row>
     <row r="87">
@@ -1551,11 +1551,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EZ_GLCpts_inferred_0</t>
+          <t>EZ_TKT1_inferred_0</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>7.162894411256191e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -1564,11 +1564,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EZ_GAPD</t>
+          <t>EZ_ADK1</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1.609232464816884e-05</v>
+        <v>1.636738824898912e-09</v>
       </c>
     </row>
     <row r="89">
@@ -1577,11 +1577,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>EZ_GLUDy</t>
+          <t>EZ_ALCD2x_inferred_0</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>7.984529441470953e-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -1590,11 +1590,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EZ_ACONTb_inferred_0</t>
+          <t>EZ_ME2_inferred_0</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>3.854841670757026e-06</v>
+        <v>3.920288378178753e-07</v>
       </c>
     </row>
     <row r="91">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EZ_ACKr_inferred_2</t>
+          <t>EZ_FUM_inferred_0</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>EZ_TKT1_inferred_0</t>
+          <t>EZ_GLUN_inferred_2</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -1629,11 +1629,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EZ_FBA_inferred_2</t>
+          <t>EZ_PYK_inferred_0</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>0</v>
+        <v>1.96794116717013e-06</v>
       </c>
     </row>
     <row r="94">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>EZ_ALCD2x_inferred_1</t>
+          <t>EZ_FUM_inferred_2</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -1655,11 +1655,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>EZ_RPI_inferred_0</t>
+          <t>EZ_FUM_inferred_1</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>0</v>
+        <v>5.775578276093036e-06</v>
       </c>
     </row>
     <row r="96">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>EZ_FBP_inferred_0</t>
+          <t>EZ_GLUSy_inferred_0</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>EZ_ACKr_inferred_0</t>
+          <t>EZ_PPS_inferred_0</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -1694,11 +1694,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>EZ_ADK1</t>
+          <t>EZ_PFK</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>0</v>
+        <v>7.923240633743083e-07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>